<commit_message>
Updating dat and adding new baseball stats
</commit_message>
<xml_diff>
--- a/backend/data/mlb/Season_Aggregated_Pitcher_Statistics.xlsx
+++ b/backend/data/mlb/Season_Aggregated_Pitcher_Statistics.xlsx
@@ -66151,61 +66151,61 @@
         <v>474</v>
       </c>
       <c r="H754">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="I754">
         <v>0</v>
       </c>
       <c r="J754">
-        <v>0</v>
+        <v>0.063</v>
       </c>
       <c r="K754">
-        <v>0</v>
+        <v>0.179</v>
       </c>
       <c r="L754">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="M754">
-        <v>0</v>
+        <v>0.062</v>
       </c>
       <c r="N754">
         <v>0</v>
       </c>
       <c r="O754">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="P754">
-        <v>0</v>
+        <v>15.8</v>
       </c>
       <c r="Q754">
-        <v>0</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="R754">
-        <v>3.12</v>
+        <v>4.12</v>
       </c>
       <c r="S754">
-        <v>7.34</v>
+        <v>6.64</v>
       </c>
       <c r="T754">
-        <v>0</v>
+        <v>28.6</v>
       </c>
       <c r="U754">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="V754">
-        <v>100</v>
+        <v>64.3</v>
       </c>
       <c r="W754">
         <v>0</v>
       </c>
       <c r="X754">
-        <v>50</v>
+        <v>14.3</v>
       </c>
       <c r="Y754">
-        <v>50</v>
+        <v>64.3</v>
       </c>
       <c r="Z754">
-        <v>0</v>
+        <v>21.4</v>
       </c>
       <c r="AA754" t="s">
         <v>405</v>
@@ -66237,58 +66237,58 @@
         <v>475</v>
       </c>
       <c r="H755">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I755">
         <v>0</v>
       </c>
       <c r="J755">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="K755">
-        <v>0</v>
+        <v>0.449</v>
       </c>
       <c r="L755">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M755">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="N755">
         <v>0</v>
       </c>
       <c r="O755">
-        <v>100</v>
+        <v>16.7</v>
       </c>
       <c r="P755">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="Q755">
-        <v>0</v>
+        <v>0.333</v>
       </c>
       <c r="R755">
-        <v>-2.88</v>
+        <v>7.12</v>
       </c>
       <c r="S755">
-        <v>-2.88</v>
+        <v>8.52</v>
       </c>
       <c r="T755">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="U755">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="V755">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="W755">
         <v>0</v>
       </c>
       <c r="X755">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="Y755">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="Z755">
         <v>0</v>
@@ -66323,61 +66323,61 @@
         <v>474</v>
       </c>
       <c r="H756">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I756">
         <v>4</v>
       </c>
       <c r="J756">
-        <v>0.239</v>
+        <v>0.248</v>
       </c>
       <c r="K756">
-        <v>0.31</v>
+        <v>0.318</v>
       </c>
       <c r="L756">
-        <v>0.364</v>
+        <v>0.377</v>
       </c>
       <c r="M756">
-        <v>0.125</v>
+        <v>0.129</v>
       </c>
       <c r="N756">
         <v>0</v>
       </c>
       <c r="O756">
-        <v>22.9</v>
+        <v>22.4</v>
       </c>
       <c r="P756">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="Q756">
-        <v>0.296</v>
+        <v>0.306</v>
       </c>
       <c r="R756">
-        <v>4.18</v>
+        <v>4.17</v>
       </c>
       <c r="S756">
-        <v>4.21</v>
+        <v>4.2</v>
       </c>
       <c r="T756">
-        <v>40</v>
+        <v>40.7</v>
       </c>
       <c r="U756">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="V756">
-        <v>35.8</v>
+        <v>34.9</v>
       </c>
       <c r="W756">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="X756">
-        <v>19</v>
+        <v>19.3</v>
       </c>
       <c r="Y756">
-        <v>56.1</v>
+        <v>56.4</v>
       </c>
       <c r="Z756">
-        <v>24.9</v>
+        <v>24.3</v>
       </c>
       <c r="AA756" t="s">
         <v>406</v>
@@ -66409,61 +66409,61 @@
         <v>475</v>
       </c>
       <c r="H757">
-        <v>412</v>
+        <v>433</v>
       </c>
       <c r="I757">
         <v>11</v>
       </c>
       <c r="J757">
-        <v>0.224</v>
+        <v>0.219</v>
       </c>
       <c r="K757">
-        <v>0.3</v>
+        <v>0.294</v>
       </c>
       <c r="L757">
-        <v>0.372</v>
+        <v>0.362</v>
       </c>
       <c r="M757">
-        <v>0.149</v>
+        <v>0.143</v>
       </c>
       <c r="N757">
         <v>0</v>
       </c>
       <c r="O757">
-        <v>26.7</v>
+        <v>26.3</v>
       </c>
       <c r="P757">
+        <v>10.1</v>
+      </c>
+      <c r="Q757">
+        <v>0.277</v>
+      </c>
+      <c r="R757">
+        <v>3.63</v>
+      </c>
+      <c r="S757">
+        <v>3.76</v>
+      </c>
+      <c r="T757">
+        <v>42.6</v>
+      </c>
+      <c r="U757">
+        <v>18.8</v>
+      </c>
+      <c r="V757">
+        <v>38.6</v>
+      </c>
+      <c r="W757">
         <v>10.4</v>
       </c>
-      <c r="Q757">
-        <v>0.284</v>
-      </c>
-      <c r="R757">
-        <v>3.72</v>
-      </c>
-      <c r="S757">
-        <v>3.77</v>
-      </c>
-      <c r="T757">
-        <v>42.2</v>
-      </c>
-      <c r="U757">
-        <v>19.1</v>
-      </c>
-      <c r="V757">
-        <v>38.7</v>
-      </c>
-      <c r="W757">
-        <v>11</v>
-      </c>
       <c r="X757">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="Y757">
-        <v>53.1</v>
+        <v>54.3</v>
       </c>
       <c r="Z757">
-        <v>34.1</v>
+        <v>32.5</v>
       </c>
       <c r="AA757" t="s">
         <v>406</v>
@@ -66495,61 +66495,61 @@
         <v>474</v>
       </c>
       <c r="H758">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I758">
         <v>3</v>
       </c>
       <c r="J758">
-        <v>0.246</v>
+        <v>0.234</v>
       </c>
       <c r="K758">
-        <v>0.302</v>
+        <v>0.288</v>
       </c>
       <c r="L758">
-        <v>0.412</v>
+        <v>0.394</v>
       </c>
       <c r="M758">
-        <v>0.167</v>
+        <v>0.16</v>
       </c>
       <c r="N758">
         <v>0</v>
       </c>
       <c r="O758">
-        <v>36</v>
+        <v>34.4</v>
       </c>
       <c r="P758">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="Q758">
-        <v>0.356</v>
+        <v>0.321</v>
       </c>
       <c r="R758">
-        <v>3.34</v>
+        <v>3.39</v>
       </c>
       <c r="S758">
-        <v>2.02</v>
+        <v>2.2</v>
       </c>
       <c r="T758">
-        <v>41.5</v>
+        <v>43.7</v>
       </c>
       <c r="U758">
-        <v>27.2</v>
+        <v>24.1</v>
       </c>
       <c r="V758">
-        <v>31.2</v>
+        <v>32.1</v>
       </c>
       <c r="W758">
-        <v>13.6</v>
+        <v>13</v>
       </c>
       <c r="X758">
-        <v>30.1</v>
+        <v>27.3</v>
       </c>
       <c r="Y758">
-        <v>43.8</v>
+        <v>48.6</v>
       </c>
       <c r="Z758">
-        <v>26.2</v>
+        <v>24.1</v>
       </c>
       <c r="AA758" t="s">
         <v>407</v>
@@ -66581,61 +66581,61 @@
         <v>475</v>
       </c>
       <c r="H759">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="I759">
         <v>10</v>
       </c>
       <c r="J759">
-        <v>0.245</v>
+        <v>0.232</v>
       </c>
       <c r="K759">
-        <v>0.317</v>
+        <v>0.305</v>
       </c>
       <c r="L759">
-        <v>0.422</v>
+        <v>0.398</v>
       </c>
       <c r="M759">
-        <v>0.177</v>
+        <v>0.165</v>
       </c>
       <c r="N759">
         <v>0</v>
       </c>
       <c r="O759">
-        <v>22.7</v>
+        <v>24.3</v>
       </c>
       <c r="P759">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="Q759">
-        <v>0.281</v>
+        <v>0.273</v>
       </c>
       <c r="R759">
-        <v>4.28</v>
+        <v>4.06</v>
       </c>
       <c r="S759">
-        <v>3.86</v>
+        <v>3.71</v>
       </c>
       <c r="T759">
-        <v>42.5</v>
+        <v>43.9</v>
       </c>
       <c r="U759">
-        <v>18.4</v>
+        <v>17.5</v>
       </c>
       <c r="V759">
-        <v>39.2</v>
+        <v>38.6</v>
       </c>
       <c r="W759">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="X759">
-        <v>17.7</v>
+        <v>17</v>
       </c>
       <c r="Y759">
-        <v>51.4</v>
+        <v>52.4</v>
       </c>
       <c r="Z759">
-        <v>30.9</v>
+        <v>30.6</v>
       </c>
       <c r="AA759" t="s">
         <v>407</v>
@@ -66667,61 +66667,61 @@
         <v>474</v>
       </c>
       <c r="H760">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="I760">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J760">
-        <v>0.297</v>
+        <v>0.285</v>
       </c>
       <c r="K760">
-        <v>0.38</v>
+        <v>0.373</v>
       </c>
       <c r="L760">
-        <v>0.518</v>
+        <v>0.506</v>
       </c>
       <c r="M760">
-        <v>0.221</v>
+        <v>0.22</v>
       </c>
       <c r="N760">
         <v>0</v>
       </c>
       <c r="O760">
+        <v>14.8</v>
+      </c>
+      <c r="P760">
+        <v>10.5</v>
+      </c>
+      <c r="Q760">
+        <v>0.299</v>
+      </c>
+      <c r="R760">
+        <v>5.76</v>
+      </c>
+      <c r="S760">
+        <v>5.34</v>
+      </c>
+      <c r="T760">
+        <v>40.3</v>
+      </c>
+      <c r="U760">
+        <v>16.9</v>
+      </c>
+      <c r="V760">
+        <v>42.7</v>
+      </c>
+      <c r="W760">
         <v>14.5</v>
       </c>
-      <c r="P760">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="Q760">
-        <v>0.315</v>
-      </c>
-      <c r="R760">
-        <v>5.65</v>
-      </c>
-      <c r="S760">
-        <v>5.22</v>
-      </c>
-      <c r="T760">
-        <v>42.1</v>
-      </c>
-      <c r="U760">
-        <v>17.6</v>
-      </c>
-      <c r="V760">
-        <v>40.4</v>
-      </c>
-      <c r="W760">
-        <v>14.7</v>
-      </c>
       <c r="X760">
-        <v>15.2</v>
+        <v>15.9</v>
       </c>
       <c r="Y760">
-        <v>52.2</v>
+        <v>52.3</v>
       </c>
       <c r="Z760">
-        <v>32.7</v>
+        <v>31.8</v>
       </c>
       <c r="AA760" t="s">
         <v>408</v>
@@ -66753,61 +66753,61 @@
         <v>475</v>
       </c>
       <c r="H761">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I761">
         <v>7</v>
       </c>
       <c r="J761">
-        <v>0.268</v>
+        <v>0.265</v>
       </c>
       <c r="K761">
-        <v>0.333</v>
+        <v>0.331</v>
       </c>
       <c r="L761">
-        <v>0.457</v>
+        <v>0.455</v>
       </c>
       <c r="M761">
-        <v>0.189</v>
+        <v>0.19</v>
       </c>
       <c r="N761">
         <v>0</v>
       </c>
       <c r="O761">
-        <v>21.1</v>
+        <v>21.7</v>
       </c>
       <c r="P761">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="Q761">
-        <v>0.295</v>
+        <v>0.297</v>
       </c>
       <c r="R761">
-        <v>4.7</v>
+        <v>4.52</v>
       </c>
       <c r="S761">
-        <v>4.07</v>
+        <v>3.95</v>
       </c>
       <c r="T761">
-        <v>44.3</v>
+        <v>44</v>
       </c>
       <c r="U761">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="V761">
-        <v>39.5</v>
+        <v>39.4</v>
       </c>
       <c r="W761">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="X761">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="Y761">
-        <v>58.9</v>
+        <v>60</v>
       </c>
       <c r="Z761">
-        <v>29.5</v>
+        <v>28.7</v>
       </c>
       <c r="AA761" t="s">
         <v>408</v>
@@ -66839,61 +66839,61 @@
         <v>474</v>
       </c>
       <c r="H762">
-        <v>422</v>
+        <v>434</v>
       </c>
       <c r="I762">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J762">
-        <v>0.23</v>
+        <v>0.231</v>
       </c>
       <c r="K762">
-        <v>0.291</v>
+        <v>0.293</v>
       </c>
       <c r="L762">
-        <v>0.375</v>
+        <v>0.38</v>
       </c>
       <c r="M762">
-        <v>0.145</v>
+        <v>0.148</v>
       </c>
       <c r="N762">
         <v>0</v>
       </c>
       <c r="O762">
-        <v>24.9</v>
+        <v>24.4</v>
       </c>
       <c r="P762">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="Q762">
-        <v>0.275</v>
+        <v>0.273</v>
       </c>
       <c r="R762">
-        <v>3.9</v>
+        <v>4.02</v>
       </c>
       <c r="S762">
-        <v>3.58</v>
+        <v>3.63</v>
       </c>
       <c r="T762">
-        <v>44</v>
+        <v>44.2</v>
       </c>
       <c r="U762">
-        <v>18.1</v>
+        <v>17.8</v>
       </c>
       <c r="V762">
-        <v>37.9</v>
+        <v>38</v>
       </c>
       <c r="W762">
-        <v>14.4</v>
+        <v>14.7</v>
       </c>
       <c r="X762">
-        <v>10.9</v>
+        <v>11.5</v>
       </c>
       <c r="Y762">
-        <v>55.8</v>
+        <v>55.9</v>
       </c>
       <c r="Z762">
-        <v>33.3</v>
+        <v>32.6</v>
       </c>
       <c r="AA762" t="s">
         <v>409</v>
@@ -66925,61 +66925,61 @@
         <v>475</v>
       </c>
       <c r="H763">
-        <v>310</v>
+        <v>321</v>
       </c>
       <c r="I763">
         <v>9</v>
       </c>
       <c r="J763">
-        <v>0.187</v>
+        <v>0.184</v>
       </c>
       <c r="K763">
-        <v>0.233</v>
+        <v>0.228</v>
       </c>
       <c r="L763">
-        <v>0.3</v>
+        <v>0.293</v>
       </c>
       <c r="M763">
-        <v>0.113</v>
+        <v>0.109</v>
       </c>
       <c r="N763">
         <v>0</v>
       </c>
       <c r="O763">
-        <v>19</v>
+        <v>19.9</v>
       </c>
       <c r="P763">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="Q763">
-        <v>0.204</v>
+        <v>0.202</v>
       </c>
       <c r="R763">
-        <v>3.7</v>
+        <v>3.58</v>
       </c>
       <c r="S763">
-        <v>3.55</v>
+        <v>3.48</v>
       </c>
       <c r="T763">
-        <v>55.9</v>
+        <v>55.2</v>
       </c>
       <c r="U763">
         <v>14.3</v>
       </c>
       <c r="V763">
-        <v>29.8</v>
+        <v>30.5</v>
       </c>
       <c r="W763">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="X763">
-        <v>13.1</v>
+        <v>13.7</v>
       </c>
       <c r="Y763">
-        <v>55.4</v>
+        <v>55.2</v>
       </c>
       <c r="Z763">
-        <v>31.5</v>
+        <v>31.1</v>
       </c>
       <c r="AA763" t="s">
         <v>409</v>
@@ -67011,22 +67011,22 @@
         <v>474</v>
       </c>
       <c r="H764">
-        <v>475</v>
+        <v>493</v>
       </c>
       <c r="I764">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J764">
-        <v>0.198</v>
+        <v>0.21</v>
       </c>
       <c r="K764">
-        <v>0.256</v>
+        <v>0.268</v>
       </c>
       <c r="L764">
-        <v>0.332</v>
+        <v>0.353</v>
       </c>
       <c r="M764">
-        <v>0.134</v>
+        <v>0.143</v>
       </c>
       <c r="N764">
         <v>0</v>
@@ -67035,37 +67035,37 @@
         <v>22.3</v>
       </c>
       <c r="P764">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="Q764">
-        <v>0.232</v>
+        <v>0.246</v>
       </c>
       <c r="R764">
-        <v>3.33</v>
+        <v>3.36</v>
       </c>
       <c r="S764">
-        <v>3.87</v>
+        <v>3.84</v>
       </c>
       <c r="T764">
-        <v>38.5</v>
+        <v>38.2</v>
       </c>
       <c r="U764">
-        <v>19.9</v>
+        <v>20.5</v>
       </c>
       <c r="V764">
-        <v>41.6</v>
+        <v>41.3</v>
       </c>
       <c r="W764">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="X764">
-        <v>16</v>
+        <v>16.8</v>
       </c>
       <c r="Y764">
-        <v>51.9</v>
+        <v>51.5</v>
       </c>
       <c r="Z764">
-        <v>32</v>
+        <v>31.6</v>
       </c>
       <c r="AA764" t="s">
         <v>410</v>
@@ -67097,58 +67097,58 @@
         <v>475</v>
       </c>
       <c r="H765">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="I765">
         <v>15</v>
       </c>
       <c r="J765">
-        <v>0.233</v>
+        <v>0.232</v>
       </c>
       <c r="K765">
-        <v>0.286</v>
+        <v>0.284</v>
       </c>
       <c r="L765">
-        <v>0.374</v>
+        <v>0.372</v>
       </c>
       <c r="M765">
-        <v>0.141</v>
+        <v>0.14</v>
       </c>
       <c r="N765">
         <v>0</v>
       </c>
       <c r="O765">
-        <v>26</v>
+        <v>25.8</v>
       </c>
       <c r="P765">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="Q765">
-        <v>0.288</v>
+        <v>0.287</v>
       </c>
       <c r="R765">
-        <v>3.43</v>
+        <v>3.41</v>
       </c>
       <c r="S765">
-        <v>3.54</v>
+        <v>3.53</v>
       </c>
       <c r="T765">
-        <v>35.9</v>
+        <v>36.2</v>
       </c>
       <c r="U765">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="V765">
-        <v>42.1</v>
+        <v>41.8</v>
       </c>
       <c r="W765">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="X765">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="Y765">
-        <v>45.9</v>
+        <v>46.1</v>
       </c>
       <c r="Z765">
         <v>39.5</v>
@@ -67183,61 +67183,61 @@
         <v>474</v>
       </c>
       <c r="H766">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="I766">
         <v>10</v>
       </c>
       <c r="J766">
-        <v>0.261</v>
+        <v>0.254</v>
       </c>
       <c r="K766">
-        <v>0.345</v>
+        <v>0.337</v>
       </c>
       <c r="L766">
-        <v>0.441</v>
+        <v>0.428</v>
       </c>
       <c r="M766">
-        <v>0.18</v>
+        <v>0.173</v>
       </c>
       <c r="N766">
         <v>0</v>
       </c>
       <c r="O766">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="P766">
         <v>8.1</v>
       </c>
       <c r="Q766">
-        <v>0.322</v>
+        <v>0.31</v>
       </c>
       <c r="R766">
-        <v>4.3</v>
+        <v>4.26</v>
       </c>
       <c r="S766">
-        <v>3.98</v>
+        <v>3.97</v>
       </c>
       <c r="T766">
-        <v>43.1</v>
+        <v>44.4</v>
       </c>
       <c r="U766">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="V766">
-        <v>36.5</v>
+        <v>35.3</v>
       </c>
       <c r="W766">
-        <v>13.9</v>
+        <v>13.6</v>
       </c>
       <c r="X766">
-        <v>11.1</v>
+        <v>10.6</v>
       </c>
       <c r="Y766">
-        <v>52.2</v>
+        <v>53.1</v>
       </c>
       <c r="Z766">
-        <v>36.7</v>
+        <v>36.3</v>
       </c>
       <c r="AA766" t="s">
         <v>411</v>
@@ -67269,7 +67269,7 @@
         <v>475</v>
       </c>
       <c r="H767">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="I767">
         <v>6</v>
@@ -67278,52 +67278,52 @@
         <v>0.205</v>
       </c>
       <c r="K767">
-        <v>0.279</v>
+        <v>0.275</v>
       </c>
       <c r="L767">
-        <v>0.333</v>
+        <v>0.327</v>
       </c>
       <c r="M767">
-        <v>0.128</v>
+        <v>0.122</v>
       </c>
       <c r="N767">
         <v>0</v>
       </c>
       <c r="O767">
-        <v>26.4</v>
+        <v>26.9</v>
       </c>
       <c r="P767">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="Q767">
-        <v>0.259</v>
+        <v>0.262</v>
       </c>
       <c r="R767">
-        <v>3.59</v>
+        <v>3.44</v>
       </c>
       <c r="S767">
-        <v>3.98</v>
+        <v>3.84</v>
       </c>
       <c r="T767">
-        <v>41.2</v>
+        <v>41.5</v>
       </c>
       <c r="U767">
-        <v>13.5</v>
+        <v>14.3</v>
       </c>
       <c r="V767">
-        <v>45.3</v>
+        <v>44.2</v>
       </c>
       <c r="W767">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="X767">
-        <v>16.9</v>
+        <v>16.2</v>
       </c>
       <c r="Y767">
-        <v>52.3</v>
+        <v>52.9</v>
       </c>
       <c r="Z767">
-        <v>30.9</v>
+        <v>31</v>
       </c>
       <c r="AA767" t="s">
         <v>411</v>
@@ -67527,61 +67527,61 @@
         <v>474</v>
       </c>
       <c r="H770">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="I770">
         <v>10</v>
       </c>
       <c r="J770">
-        <v>0.247</v>
+        <v>0.244</v>
       </c>
       <c r="K770">
-        <v>0.302</v>
+        <v>0.299</v>
       </c>
       <c r="L770">
-        <v>0.369</v>
+        <v>0.364</v>
       </c>
       <c r="M770">
-        <v>0.123</v>
+        <v>0.12</v>
       </c>
       <c r="N770">
         <v>0</v>
       </c>
       <c r="O770">
-        <v>23.5</v>
+        <v>23.8</v>
       </c>
       <c r="P770">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="Q770">
-        <v>0.306</v>
+        <v>0.304</v>
       </c>
       <c r="R770">
-        <v>3.65</v>
+        <v>3.58</v>
       </c>
       <c r="S770">
-        <v>3.62</v>
+        <v>3.56</v>
       </c>
       <c r="T770">
-        <v>49.9</v>
+        <v>50.1</v>
       </c>
       <c r="U770">
         <v>17.9</v>
       </c>
       <c r="V770">
-        <v>32.3</v>
+        <v>32.1</v>
       </c>
       <c r="W770">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="X770">
-        <v>13.5</v>
+        <v>13.2</v>
       </c>
       <c r="Y770">
-        <v>53.5</v>
+        <v>53.3</v>
       </c>
       <c r="Z770">
-        <v>33</v>
+        <v>33.5</v>
       </c>
       <c r="AA770" t="s">
         <v>413</v>
@@ -67613,61 +67613,61 @@
         <v>475</v>
       </c>
       <c r="H771">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="I771">
         <v>9</v>
       </c>
       <c r="J771">
-        <v>0.249</v>
+        <v>0.257</v>
       </c>
       <c r="K771">
-        <v>0.285</v>
+        <v>0.293</v>
       </c>
       <c r="L771">
-        <v>0.377</v>
+        <v>0.38</v>
       </c>
       <c r="M771">
-        <v>0.127</v>
+        <v>0.123</v>
       </c>
       <c r="N771">
         <v>0</v>
       </c>
       <c r="O771">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="P771">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="Q771">
-        <v>0.305</v>
+        <v>0.318</v>
       </c>
       <c r="R771">
+        <v>3.06</v>
+      </c>
+      <c r="S771">
         <v>3.08</v>
       </c>
-      <c r="S771">
-        <v>3.1</v>
-      </c>
       <c r="T771">
-        <v>45.6</v>
+        <v>45.7</v>
       </c>
       <c r="U771">
-        <v>20.4</v>
+        <v>21.6</v>
       </c>
       <c r="V771">
-        <v>34</v>
+        <v>32.7</v>
       </c>
       <c r="W771">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="X771">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="Y771">
         <v>58.2</v>
       </c>
       <c r="Z771">
-        <v>30.8</v>
+        <v>31.2</v>
       </c>
       <c r="AA771" t="s">
         <v>413</v>
@@ -67699,61 +67699,61 @@
         <v>474</v>
       </c>
       <c r="H772">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="I772">
         <v>0</v>
       </c>
       <c r="J772">
-        <v>0.14</v>
+        <v>0.129</v>
       </c>
       <c r="K772">
-        <v>0.23</v>
+        <v>0.201</v>
       </c>
       <c r="L772">
-        <v>0.16</v>
+        <v>0.143</v>
       </c>
       <c r="M772">
-        <v>0.02</v>
+        <v>0.014</v>
       </c>
       <c r="N772">
         <v>0</v>
       </c>
       <c r="O772">
-        <v>30</v>
+        <v>28.4</v>
       </c>
       <c r="P772">
-        <v>15</v>
+        <v>12.3</v>
       </c>
       <c r="Q772">
-        <v>0.219</v>
+        <v>0.191</v>
       </c>
       <c r="R772">
-        <v>2.7</v>
+        <v>2.49</v>
       </c>
       <c r="S772">
-        <v>3.97</v>
+        <v>3.71</v>
       </c>
       <c r="T772">
-        <v>45.2</v>
+        <v>47.8</v>
       </c>
       <c r="U772">
-        <v>12.9</v>
+        <v>13</v>
       </c>
       <c r="V772">
-        <v>41.9</v>
+        <v>39.1</v>
       </c>
       <c r="W772">
         <v>0</v>
       </c>
       <c r="X772">
-        <v>15.6</v>
+        <v>12.8</v>
       </c>
       <c r="Y772">
-        <v>68.8</v>
+        <v>63.8</v>
       </c>
       <c r="Z772">
-        <v>15.6</v>
+        <v>23.4</v>
       </c>
       <c r="AA772" t="s">
         <v>414</v>
@@ -67785,61 +67785,61 @@
         <v>475</v>
       </c>
       <c r="H773">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="I773">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J773">
-        <v>0.267</v>
+        <v>0.333</v>
       </c>
       <c r="K773">
-        <v>0.318</v>
+        <v>0.392</v>
       </c>
       <c r="L773">
-        <v>0.367</v>
+        <v>0.5</v>
       </c>
       <c r="M773">
-        <v>0.1</v>
+        <v>0.167</v>
       </c>
       <c r="N773">
         <v>0</v>
       </c>
       <c r="O773">
-        <v>15.2</v>
+        <v>15.4</v>
       </c>
       <c r="P773">
-        <v>6.1</v>
+        <v>5.1</v>
       </c>
       <c r="Q773">
-        <v>0.32</v>
+        <v>0.379</v>
       </c>
       <c r="R773">
-        <v>2.99</v>
+        <v>4.27</v>
       </c>
       <c r="S773">
-        <v>4.22</v>
+        <v>4.07</v>
       </c>
       <c r="T773">
-        <v>44</v>
+        <v>43.3</v>
       </c>
       <c r="U773">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="V773">
-        <v>28</v>
+        <v>26.7</v>
       </c>
       <c r="W773">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="X773">
-        <v>8</v>
+        <v>6.7</v>
       </c>
       <c r="Y773">
         <v>60</v>
       </c>
       <c r="Z773">
-        <v>32</v>
+        <v>33.3</v>
       </c>
       <c r="AA773" t="s">
         <v>414</v>
@@ -67871,61 +67871,61 @@
         <v>474</v>
       </c>
       <c r="H774">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="I774">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J774">
-        <v>0.321</v>
+        <v>0.341</v>
       </c>
       <c r="K774">
-        <v>0.363</v>
+        <v>0.4</v>
       </c>
       <c r="L774">
-        <v>0.428</v>
+        <v>0.509</v>
       </c>
       <c r="M774">
-        <v>0.107</v>
+        <v>0.167</v>
       </c>
       <c r="N774">
         <v>0</v>
       </c>
       <c r="O774">
-        <v>21.9</v>
+        <v>19.6</v>
       </c>
       <c r="P774">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="Q774">
-        <v>0.375</v>
+        <v>0.387</v>
       </c>
       <c r="R774">
-        <v>4.34</v>
+        <v>5.35</v>
       </c>
       <c r="S774">
-        <v>3.26</v>
+        <v>3.42</v>
       </c>
       <c r="T774">
-        <v>41.6</v>
+        <v>53.3</v>
       </c>
       <c r="U774">
-        <v>37.2</v>
+        <v>27.9</v>
       </c>
       <c r="V774">
-        <v>21.4</v>
+        <v>18.9</v>
       </c>
       <c r="W774">
-        <v>12.5</v>
+        <v>23.9</v>
       </c>
       <c r="X774">
-        <v>12.5</v>
+        <v>15.1</v>
       </c>
       <c r="Y774">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="Z774">
-        <v>39.6</v>
+        <v>36.8</v>
       </c>
       <c r="AA774" t="s">
         <v>415</v>
@@ -67957,61 +67957,61 @@
         <v>475</v>
       </c>
       <c r="H775">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="I775">
         <v>1</v>
       </c>
       <c r="J775">
-        <v>0.116</v>
+        <v>0.159</v>
       </c>
       <c r="K775">
-        <v>0.131</v>
+        <v>0.18</v>
       </c>
       <c r="L775">
-        <v>0.192</v>
+        <v>0.237</v>
       </c>
       <c r="M775">
-        <v>0.077</v>
+        <v>0.079</v>
       </c>
       <c r="N775">
         <v>0</v>
       </c>
       <c r="O775">
-        <v>28.9</v>
+        <v>26.6</v>
       </c>
       <c r="P775">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="Q775">
-        <v>0.138</v>
+        <v>0.2</v>
       </c>
       <c r="R775">
-        <v>2.07</v>
+        <v>2.13</v>
       </c>
       <c r="S775">
-        <v>2.1</v>
+        <v>2.25</v>
       </c>
       <c r="T775">
-        <v>65.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="U775">
-        <v>10.8</v>
+        <v>13</v>
       </c>
       <c r="V775">
-        <v>24.1</v>
+        <v>21.7</v>
       </c>
       <c r="W775">
-        <v>8.699999999999999</v>
+        <v>7</v>
       </c>
       <c r="X775">
-        <v>16.4</v>
+        <v>13</v>
       </c>
       <c r="Y775">
-        <v>43.3</v>
+        <v>52.2</v>
       </c>
       <c r="Z775">
-        <v>40.4</v>
+        <v>34.7</v>
       </c>
       <c r="AA775" t="s">
         <v>415</v>
@@ -68043,61 +68043,61 @@
         <v>474</v>
       </c>
       <c r="H776">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="I776">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J776">
-        <v>0.246</v>
+        <v>0.25</v>
       </c>
       <c r="K776">
-        <v>0.364</v>
+        <v>0.367</v>
       </c>
       <c r="L776">
-        <v>0.449</v>
+        <v>0.461</v>
       </c>
       <c r="M776">
-        <v>0.204</v>
+        <v>0.211</v>
       </c>
       <c r="N776">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O776">
-        <v>18.2</v>
+        <v>17.9</v>
       </c>
       <c r="P776">
-        <v>15.2</v>
+        <v>14.5</v>
       </c>
       <c r="Q776">
         <v>0.258</v>
       </c>
       <c r="R776">
-        <v>6.45</v>
+        <v>6.56</v>
       </c>
       <c r="S776">
-        <v>5.9</v>
+        <v>5.85</v>
       </c>
       <c r="T776">
-        <v>29.7</v>
+        <v>29.4</v>
       </c>
       <c r="U776">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="V776">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="W776">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="X776">
-        <v>13.4</v>
+        <v>12.6</v>
       </c>
       <c r="Y776">
-        <v>54.4</v>
+        <v>55.7</v>
       </c>
       <c r="Z776">
-        <v>32.2</v>
+        <v>31.7</v>
       </c>
       <c r="AA776" t="s">
         <v>416</v>
@@ -68129,7 +68129,7 @@
         <v>475</v>
       </c>
       <c r="H777">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="I777">
         <v>6</v>
@@ -68138,52 +68138,52 @@
         <v>0.257</v>
       </c>
       <c r="K777">
-        <v>0.373</v>
+        <v>0.368</v>
       </c>
       <c r="L777">
-        <v>0.506</v>
+        <v>0.489</v>
       </c>
       <c r="M777">
-        <v>0.249</v>
+        <v>0.232</v>
       </c>
       <c r="N777">
         <v>0</v>
       </c>
       <c r="O777">
-        <v>18.4</v>
+        <v>19.4</v>
       </c>
       <c r="P777">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="Q777">
-        <v>0.276</v>
+        <v>0.286</v>
       </c>
       <c r="R777">
-        <v>6.06</v>
+        <v>5.69</v>
       </c>
       <c r="S777">
-        <v>4.64</v>
+        <v>4.46</v>
       </c>
       <c r="T777">
-        <v>50</v>
+        <v>52.3</v>
       </c>
       <c r="U777">
-        <v>18.4</v>
+        <v>17.8</v>
       </c>
       <c r="V777">
-        <v>31.6</v>
+        <v>29.9</v>
       </c>
       <c r="W777">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="X777">
-        <v>15.1</v>
+        <v>13.7</v>
       </c>
       <c r="Y777">
-        <v>54.4</v>
+        <v>55.1</v>
       </c>
       <c r="Z777">
-        <v>30.6</v>
+        <v>31.3</v>
       </c>
       <c r="AA777" t="s">
         <v>416</v>

</xml_diff>